<commit_message>
Graduate tanks T0182 (30 fish) and T0183 (12 fish) from Cross C0072 (AB T128)
</commit_message>
<xml_diff>
--- a/FishNET_Colony_Analytics_Report.xlsx
+++ b/FishNET_Colony_Analytics_Report.xlsx
@@ -551,7 +551,7 @@
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
   </cols>
@@ -575,21 +575,21 @@
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Total Recorded Tanks
-180</t>
+183</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Active Holding Tanks
-117</t>
+120</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Total Active Fish
-1251</t>
+1293</t>
         </is>
       </c>
       <c r="F4" s="4" t="n"/>
@@ -848,13 +848,13 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C13" s="8" t="n">
         <v>12</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="E13" s="8" t="n">
         <v>0</v>
@@ -875,7 +875,7 @@
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>Extinct / Inactive</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>9.6%</t>
+          <t>9.3%</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>36.9%</t>
+          <t>35.7%</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>9.0%</t>
+          <t>8.7%</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>20.2%</t>
+          <t>19.6%</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>24.2%</t>
+          <t>23.4%</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -1316,13 +1316,13 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>12</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="E9" s="8" t="n">
         <v>0</v>
@@ -1343,12 +1343,12 @@
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>Extinct / Inactive</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>No active tanks in facility</t>
+          <t>Healthy colony size and demographics</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M121"/>
+  <dimension ref="A1:M124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1374,7 +1374,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
@@ -8363,6 +8363,149 @@
       <c r="M121" s="10" t="inlineStr">
         <is>
           <t>Normal active holding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="11" t="inlineStr"/>
+      <c r="B122" s="11" t="inlineStr">
+        <is>
+          <t>Adult/Active</t>
+        </is>
+      </c>
+      <c r="C122" s="10" t="inlineStr"/>
+      <c r="D122" s="11" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E122" s="11" t="inlineStr"/>
+      <c r="F122" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G122" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I122" s="11" t="inlineStr"/>
+      <c r="J122" s="11" t="inlineStr"/>
+      <c r="K122" s="11" t="n"/>
+      <c r="L122" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M122" s="10" t="inlineStr">
+        <is>
+          <t>Inactive or No turnover date set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="11" t="inlineStr">
+        <is>
+          <t>10-08-26</t>
+        </is>
+      </c>
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>Adult/Active</t>
+        </is>
+      </c>
+      <c r="C123" s="10" t="inlineStr"/>
+      <c r="D123" s="11" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E123" s="11" t="inlineStr">
+        <is>
+          <t>Wt (AB)</t>
+        </is>
+      </c>
+      <c r="F123" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="G123" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H123" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I123" s="11" t="inlineStr">
+        <is>
+          <t>Huseyin Cagatay Yalcin</t>
+        </is>
+      </c>
+      <c r="J123" s="11" t="inlineStr">
+        <is>
+          <t>AB T128</t>
+        </is>
+      </c>
+      <c r="K123" s="11" t="n"/>
+      <c r="L123" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M123" s="10" t="inlineStr">
+        <is>
+          <t>Inactive or No turnover date set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="11" t="inlineStr">
+        <is>
+          <t>10-08-26</t>
+        </is>
+      </c>
+      <c r="B124" s="11" t="inlineStr">
+        <is>
+          <t>Adult/Active</t>
+        </is>
+      </c>
+      <c r="C124" s="10" t="inlineStr"/>
+      <c r="D124" s="11" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E124" s="11" t="inlineStr">
+        <is>
+          <t>Wt (AB)</t>
+        </is>
+      </c>
+      <c r="F124" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="G124" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I124" s="11" t="inlineStr">
+        <is>
+          <t>Huseyin Cagatay Yalcin</t>
+        </is>
+      </c>
+      <c r="J124" s="11" t="inlineStr">
+        <is>
+          <t>AB T128</t>
+        </is>
+      </c>
+      <c r="K124" s="11" t="n"/>
+      <c r="L124" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M124" s="10" t="inlineStr">
+        <is>
+          <t>Inactive or No turnover date set.</t>
         </is>
       </c>
     </row>
@@ -8377,7 +8520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K184"/>
+  <dimension ref="A1:K187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -16305,6 +16448,97 @@
         </is>
       </c>
     </row>
+    <row r="185">
+      <c r="A185" s="11" t="inlineStr"/>
+      <c r="B185" s="11" t="inlineStr"/>
+      <c r="C185" s="11" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D185" s="11" t="inlineStr">
+        <is>
+          <t>F0 / Founder</t>
+        </is>
+      </c>
+      <c r="E185" s="11" t="inlineStr"/>
+      <c r="F185" s="11" t="inlineStr"/>
+      <c r="G185" s="11" t="inlineStr"/>
+      <c r="H185" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I185" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J185" s="10" t="inlineStr"/>
+      <c r="K185" s="10" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="11" t="inlineStr">
+        <is>
+          <t>10-08-26</t>
+        </is>
+      </c>
+      <c r="B186" s="11" t="inlineStr"/>
+      <c r="C186" s="11" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D186" s="11" t="inlineStr">
+        <is>
+          <t>F0 / Founder</t>
+        </is>
+      </c>
+      <c r="E186" s="11" t="inlineStr"/>
+      <c r="F186" s="11" t="inlineStr"/>
+      <c r="G186" s="11" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="H186" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I186" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J186" s="10" t="inlineStr"/>
+      <c r="K186" s="10" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="11" t="inlineStr">
+        <is>
+          <t>10-08-26</t>
+        </is>
+      </c>
+      <c r="B187" s="11" t="inlineStr"/>
+      <c r="C187" s="11" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D187" s="11" t="inlineStr">
+        <is>
+          <t>F0 / Founder</t>
+        </is>
+      </c>
+      <c r="E187" s="11" t="inlineStr"/>
+      <c r="F187" s="11" t="inlineStr"/>
+      <c r="G187" s="11" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H187" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I187" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J187" s="10" t="inlineStr"/>
+      <c r="K187" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16316,13 +16550,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
@@ -16343,7 +16577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Crosses: 64 | Tracking yields for C0001 - C0071</t>
+          <t>Total Crosses: 66 | Tracking yields for C0001 - C0071</t>
         </is>
       </c>
     </row>
@@ -16413,35 +16647,35 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>C0001</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>T0038 x T0038</t>
+          <t xml:space="preserve"> x D126</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>AB</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>02-01-2024</t>
+          <t>Huseyin Cagatay Yalcin</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H5" s="11" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I5" s="11" t="n">
         <v>0</v>
@@ -16450,46 +16684,46 @@
         <v>0</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L5" s="10" t="inlineStr">
         <is>
-          <t>T0046</t>
+          <t>10-08-26</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>C0002</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>T0011 x T0011</t>
+          <t xml:space="preserve"> x D126</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Fli</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>21-11-2023</t>
+          <t>Huseyin Cagatay Yalcin</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H6" s="11" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I6" s="11" t="n">
         <v>0</v>
@@ -16498,33 +16732,33 @@
         <v>0</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="L6" s="10" t="inlineStr">
         <is>
-          <t>T0047</t>
+          <t>10-08-26</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>C0003</t>
+          <t>C0001</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>T0012 x T0012</t>
+          <t>T0038 x T0038</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Fli</t>
+          <t>AB</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>24-09-2023</t>
+          <t>02-01-2024</t>
         </is>
       </c>
       <c r="E7" s="11" t="n">
@@ -16534,7 +16768,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H7" s="11" t="n">
         <v>0</v>
@@ -16546,81 +16780,81 @@
         <v>0</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="L7" s="10" t="inlineStr">
         <is>
-          <t>T0048</t>
+          <t>T0046</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>C0004</t>
+          <t>C0002</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>T0020 x T0020</t>
+          <t>T0011 x T0011</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Gata</t>
+          <t>Fli</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>27-02-2024</t>
+          <t>21-11-2023</t>
         </is>
       </c>
       <c r="E8" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="H8" s="11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I8" s="11" t="n">
         <v>0</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="L8" s="10" t="inlineStr">
         <is>
-          <t>T0049</t>
+          <t>T0047</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>C0005</t>
+          <t>C0003</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>T0020 x T0020</t>
+          <t>T0012 x T0012</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Gata</t>
+          <t>Fli</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>23-10-2023</t>
+          <t>24-09-2023</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
@@ -16630,7 +16864,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="H9" s="11" t="n">
         <v>0</v>
@@ -16642,18 +16876,18 @@
         <v>0</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="L9" s="10" t="inlineStr">
         <is>
-          <t>T0050</t>
+          <t>T0048</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>C0006</t>
+          <t>C0004</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
@@ -16668,55 +16902,55 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>23-11-2023</t>
+          <t>27-02-2024</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F10" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="11" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="H10" s="11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I10" s="11" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="L10" s="10" t="inlineStr">
         <is>
-          <t>T0051</t>
+          <t>T0049</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>C0007</t>
+          <t>C0005</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>T0011 x T0011</t>
+          <t>T0020 x T0020</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Fli</t>
+          <t>Gata</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>11-03-2024</t>
+          <t>23-10-2023</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
@@ -16726,7 +16960,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="H11" s="11" t="n">
         <v>0</v>
@@ -16738,33 +16972,33 @@
         <v>0</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="L11" s="10" t="inlineStr">
         <is>
-          <t>T0052</t>
+          <t>T0050</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>C0008</t>
+          <t>C0006</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>T0048 x T0048</t>
+          <t>T0020 x T0020</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Fli</t>
+          <t>Gata</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>23-09-2023</t>
+          <t>23-11-2023</t>
         </is>
       </c>
       <c r="E12" s="11" t="n">
@@ -16774,7 +17008,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="11" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H12" s="11" t="n">
         <v>0</v>
@@ -16786,18 +17020,18 @@
         <v>0</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="L12" s="10" t="inlineStr">
         <is>
-          <t>T0053</t>
+          <t>T0051</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>C0009</t>
+          <t>C0007</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
@@ -16812,189 +17046,189 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>25-08-2024</t>
+          <t>11-03-2024</t>
         </is>
       </c>
       <c r="E13" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="H13" s="11" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J13" s="11" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="L13" s="10" t="inlineStr">
         <is>
-          <t>T0054</t>
+          <t>T0052</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>C0010</t>
+          <t>C0008</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>T0027 x T0027</t>
+          <t>T0048 x T0048</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>AB</t>
+          <t>Fli</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>01-09-2024</t>
+          <t>23-09-2023</t>
         </is>
       </c>
       <c r="E14" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" s="11" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H14" s="11" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="J14" s="11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K14" s="11" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="L14" s="10" t="inlineStr">
         <is>
-          <t>T0056</t>
+          <t>T0053</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>C0011</t>
+          <t>C0009</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>T0036 x T0036</t>
+          <t>T0011 x T0011</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>AB</t>
+          <t>Fli</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>12-05-2024</t>
+          <t>25-08-2024</t>
         </is>
       </c>
       <c r="E15" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" s="11" t="n">
         <v>17</v>
       </c>
       <c r="H15" s="11" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J15" s="11" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K15" s="11" t="n">
         <v>17</v>
       </c>
       <c r="L15" s="10" t="inlineStr">
         <is>
-          <t>T0057</t>
+          <t>T0054</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>C0012</t>
+          <t>C0010</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>T0011 x T0011</t>
+          <t>T0027 x T0027</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Fli</t>
+          <t>AB</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>26-06-2023</t>
+          <t>01-09-2024</t>
         </is>
       </c>
       <c r="E16" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="11" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H16" s="11" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J16" s="11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K16" s="11" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="L16" s="10" t="inlineStr">
         <is>
-          <t>T0058</t>
+          <t>T0056</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>C0013</t>
+          <t>C0011</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>T0038 x T0038</t>
+          <t>T0036 x T0036</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
@@ -17004,7 +17238,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>31-07-2023</t>
+          <t>12-05-2024</t>
         </is>
       </c>
       <c r="E17" s="11" t="n">
@@ -17030,29 +17264,29 @@
       </c>
       <c r="L17" s="10" t="inlineStr">
         <is>
-          <t>T0063</t>
+          <t>T0057</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>C0014</t>
+          <t>C0012</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>T0038 x T0038</t>
+          <t>T0011 x T0011</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>AB</t>
+          <t>Fli</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>28-08-2023</t>
+          <t>26-06-2023</t>
         </is>
       </c>
       <c r="E18" s="11" t="n">
@@ -17062,7 +17296,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="11" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H18" s="11" t="n">
         <v>0</v>
@@ -17074,18 +17308,18 @@
         <v>0</v>
       </c>
       <c r="K18" s="11" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="L18" s="10" t="inlineStr">
         <is>
-          <t>T0037</t>
+          <t>T0058</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>C0015</t>
+          <t>C0013</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
@@ -17110,7 +17344,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="11" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="H19" s="11" t="n">
         <v>0</v>
@@ -17122,18 +17356,18 @@
         <v>0</v>
       </c>
       <c r="K19" s="11" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="L19" s="10" t="inlineStr">
         <is>
-          <t>T0039</t>
+          <t>T0063</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>C0016</t>
+          <t>C0014</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
@@ -17148,7 +17382,7 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>13-09-2023</t>
+          <t>28-08-2023</t>
         </is>
       </c>
       <c r="E20" s="11" t="n">
@@ -17158,7 +17392,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="11" t="n">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="H20" s="11" t="n">
         <v>0</v>
@@ -17170,23 +17404,23 @@
         <v>0</v>
       </c>
       <c r="K20" s="11" t="n">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="L20" s="10" t="inlineStr">
         <is>
-          <t>T0044</t>
+          <t>T0037</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>C0017</t>
+          <t>C0015</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>T0026 x T0026</t>
+          <t>T0038 x T0038</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -17196,103 +17430,103 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>30-09-2024</t>
+          <t>31-07-2023</t>
         </is>
       </c>
       <c r="E21" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G21" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H21" s="11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J21" s="11" t="n">
         <v>0</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L21" s="10" t="inlineStr">
         <is>
-          <t>T0065</t>
+          <t>T0039</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>C0024</t>
+          <t>C0016</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>T0039 x T0015</t>
+          <t>T0038 x T0038</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Casper</t>
+          <t>AB</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>03-06-2024</t>
+          <t>13-09-2023</t>
         </is>
       </c>
       <c r="E22" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" s="11" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="H22" s="11" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J22" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="L22" s="10" t="inlineStr">
         <is>
-          <t>T0066</t>
+          <t>T0044</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>C0025</t>
+          <t>C0017</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>T0015 x T0015</t>
+          <t>T0026 x T0026</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Casper</t>
+          <t>AB</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>18-11-2024</t>
+          <t>30-09-2024</t>
         </is>
       </c>
       <c r="E23" s="11" t="n">
@@ -17302,35 +17536,35 @@
         <v>1</v>
       </c>
       <c r="G23" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H23" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J23" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L23" s="10" t="inlineStr">
         <is>
-          <t>T0068</t>
+          <t>T0065</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>C0026</t>
+          <t>C0024</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>T0066 x T0059</t>
+          <t>T0039 x T0015</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
@@ -17340,7 +17574,7 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>24-12-2024</t>
+          <t>03-06-2024</t>
         </is>
       </c>
       <c r="E24" s="11" t="n">
@@ -17350,45 +17584,45 @@
         <v>1</v>
       </c>
       <c r="G24" s="11" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="H24" s="11" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K24" s="11" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="L24" s="10" t="inlineStr">
         <is>
-          <t>T0069</t>
+          <t>T0066</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>C0027</t>
+          <t>C0025</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>T0011 x T0011</t>
+          <t>T0015 x T0015</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Fli</t>
+          <t>Casper</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>12-11-2024</t>
+          <t>18-11-2024</t>
         </is>
       </c>
       <c r="E25" s="11" t="n">
@@ -17398,45 +17632,45 @@
         <v>1</v>
       </c>
       <c r="G25" s="11" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K25" s="11" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L25" s="10" t="inlineStr">
         <is>
-          <t>T0070</t>
+          <t>T0068</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>C0028</t>
+          <t>C0026</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>T0049 x T0064</t>
+          <t>T0066 x T0059</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Gata</t>
+          <t>Casper</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>17-02-2025</t>
+          <t>24-12-2024</t>
         </is>
       </c>
       <c r="E26" s="11" t="n">
@@ -17446,45 +17680,45 @@
         <v>1</v>
       </c>
       <c r="G26" s="11" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="H26" s="11" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K26" s="11" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="L26" s="10" t="inlineStr">
         <is>
-          <t>T0073</t>
+          <t>T0069</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>C0029</t>
+          <t>C0027</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>T0015 x T0015</t>
+          <t>T0011 x T0011</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Casper</t>
+          <t>Fli</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>05-03-2025</t>
+          <t>12-11-2024</t>
         </is>
       </c>
       <c r="E27" s="11" t="n">
@@ -17500,29 +17734,29 @@
         <v>7</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J27" s="11" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K27" s="11" t="n">
         <v>7</v>
       </c>
       <c r="L27" s="10" t="inlineStr">
         <is>
-          <t>T0077</t>
+          <t>T0070</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>C0030</t>
+          <t>C0028</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>T0049 x T0056</t>
+          <t>T0049 x T0064</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
@@ -17532,7 +17766,7 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>17-02-2025</t>
         </is>
       </c>
       <c r="E28" s="11" t="n">
@@ -17542,45 +17776,45 @@
         <v>1</v>
       </c>
       <c r="G28" s="11" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="H28" s="11" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="J28" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" s="11" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="L28" s="10" t="inlineStr">
         <is>
-          <t>T0079</t>
+          <t>T0073</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>C0031</t>
+          <t>C0029</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>T0056 x T0053</t>
+          <t>T0015 x T0015</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Fli</t>
+          <t>Casper</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>16-03-2025</t>
+          <t>05-03-2025</t>
         </is>
       </c>
       <c r="E29" s="11" t="n">
@@ -17596,39 +17830,39 @@
         <v>7</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J29" s="11" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K29" s="11" t="n">
         <v>7</v>
       </c>
       <c r="L29" s="10" t="inlineStr">
         <is>
-          <t>T0082</t>
+          <t>T0077</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>C0032</t>
+          <t>C0030</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>T0072 x T0072</t>
+          <t>T0049 x T0056</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Fli</t>
+          <t>Gata</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="E30" s="11" t="n">
@@ -17638,35 +17872,35 @@
         <v>1</v>
       </c>
       <c r="G30" s="11" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H30" s="11" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="I30" s="11" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="J30" s="11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K30" s="11" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="L30" s="10" t="inlineStr">
         <is>
-          <t>T0104</t>
+          <t>T0079</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>C0033</t>
+          <t>C0031</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>T0082 x T0082</t>
+          <t>T0056 x T0053</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
@@ -17676,7 +17910,7 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>20-07-2025</t>
+          <t>16-03-2025</t>
         </is>
       </c>
       <c r="E31" s="11" t="n">
@@ -17686,45 +17920,45 @@
         <v>1</v>
       </c>
       <c r="G31" s="11" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H31" s="11" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I31" s="11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J31" s="11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K31" s="11" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L31" s="10" t="inlineStr">
         <is>
-          <t>T0105</t>
+          <t>T0082</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>C0034</t>
+          <t>C0032</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>T0015 x T0067</t>
+          <t>T0072 x T0072</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Casper</t>
+          <t>Fli</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="E32" s="11" t="n">
@@ -17734,45 +17968,45 @@
         <v>1</v>
       </c>
       <c r="G32" s="11" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H32" s="11" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I32" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="J32" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="K32" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="J32" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="K32" s="11" t="n">
-        <v>7</v>
-      </c>
       <c r="L32" s="10" t="inlineStr">
         <is>
-          <t>T0107</t>
+          <t>T0104</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>C0035</t>
+          <t>C0033</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>T0015 x T0067</t>
+          <t>T0082 x T0082</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>Casper</t>
+          <t>Fli</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>20-07-2025</t>
         </is>
       </c>
       <c r="E33" s="11" t="n">
@@ -17782,35 +18016,35 @@
         <v>1</v>
       </c>
       <c r="G33" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H33" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I33" s="11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J33" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L33" s="10" t="inlineStr">
         <is>
-          <t>T0108</t>
+          <t>T0105</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>C0036</t>
+          <t>C0034</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>T0015 x T0015</t>
+          <t>T0015 x T0067</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
@@ -17820,7 +18054,7 @@
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="E34" s="11" t="n">
@@ -17830,45 +18064,45 @@
         <v>1</v>
       </c>
       <c r="G34" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="H34" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="I34" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="J34" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H34" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="I34" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="J34" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="K34" s="11" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L34" s="10" t="inlineStr">
         <is>
-          <t>T0109</t>
+          <t>T0107</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>C0037</t>
+          <t>C0035</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>T0049 x T0056</t>
+          <t>T0015 x T0067</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>Gata</t>
+          <t>Casper</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>26-02-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="E35" s="11" t="n">
@@ -17894,29 +18128,29 @@
       </c>
       <c r="L35" s="10" t="inlineStr">
         <is>
-          <t>T0110</t>
+          <t>T0108</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>C0038</t>
+          <t>C0036</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>T0073 x T0073</t>
+          <t>T0015 x T0015</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Gata</t>
+          <t>Casper</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="E36" s="11" t="n">
@@ -17926,35 +18160,35 @@
         <v>1</v>
       </c>
       <c r="G36" s="11" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="H36" s="11" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="I36" s="11" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J36" s="11" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="K36" s="11" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="L36" s="10" t="inlineStr">
         <is>
-          <t>T0111</t>
+          <t>T0109</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>C0039</t>
+          <t>C0037</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>T0073 x T0073</t>
+          <t>T0049 x T0056</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
@@ -17964,7 +18198,7 @@
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>22-06-2025</t>
+          <t>26-02-2025</t>
         </is>
       </c>
       <c r="E37" s="11" t="n">
@@ -17974,93 +18208,93 @@
         <v>1</v>
       </c>
       <c r="G37" s="11" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I37" s="11" t="n">
         <v>2</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="K37" s="11" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="L37" s="10" t="inlineStr">
         <is>
-          <t>T0112</t>
+          <t>T0110</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>C0040</t>
+          <t>C0038</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>T0069 x T0069</t>
+          <t>T0073 x T0073</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Casper</t>
+          <t>Gata</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>11-09-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="E38" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F38" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G38" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="H38" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="I38" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="J38" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="H38" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="I38" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="J38" s="11" t="n">
-        <v>2</v>
-      </c>
       <c r="K38" s="11" t="n">
-        <v>3.5</v>
+        <v>17</v>
       </c>
       <c r="L38" s="10" t="inlineStr">
         <is>
-          <t>T0114, T0115</t>
+          <t>T0111</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>C0041</t>
+          <t>C0039</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>T0093 x T0095</t>
+          <t>T0073 x T0073</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>AB</t>
+          <t>Gata</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>04-09-2025</t>
+          <t>22-06-2025</t>
         </is>
       </c>
       <c r="E39" s="11" t="n">
@@ -18070,93 +18304,93 @@
         <v>1</v>
       </c>
       <c r="G39" s="11" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="H39" s="11" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K39" s="11" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="L39" s="10" t="inlineStr">
         <is>
-          <t>T0117</t>
+          <t>T0112</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>C0042</t>
+          <t>C0040</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>T0093 x T0095</t>
+          <t>T0069 x T0069</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>AB</t>
+          <t>Casper</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>16-06-2025</t>
+          <t>11-09-2025</t>
         </is>
       </c>
       <c r="E40" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F40" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G40" s="11" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="H40" s="11" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="I40" s="11" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="J40" s="11" t="n">
         <v>2</v>
       </c>
       <c r="K40" s="11" t="n">
-        <v>21</v>
+        <v>3.5</v>
       </c>
       <c r="L40" s="10" t="inlineStr">
         <is>
-          <t>T0118</t>
+          <t>T0114, T0115</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="11" t="inlineStr">
         <is>
-          <t>C0043</t>
+          <t>C0041</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>T0049 x T0073</t>
+          <t>T0093 x T0095</t>
         </is>
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Gata</t>
+          <t>AB</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>14-10-2025</t>
+          <t>04-09-2025</t>
         </is>
       </c>
       <c r="E41" s="11" t="n">
@@ -18166,45 +18400,45 @@
         <v>1</v>
       </c>
       <c r="G41" s="11" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H41" s="11" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I41" s="11" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="J41" s="11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K41" s="11" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="L41" s="10" t="inlineStr">
         <is>
-          <t>T0120</t>
+          <t>T0117</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>C0044</t>
+          <t>C0042</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>T0015 x T0067</t>
+          <t>T0093 x T0095</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Casper</t>
+          <t>AB</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>03-07-2025</t>
+          <t>16-06-2025</t>
         </is>
       </c>
       <c r="E42" s="11" t="n">
@@ -18214,45 +18448,45 @@
         <v>1</v>
       </c>
       <c r="G42" s="11" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H42" s="11" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="J42" s="11" t="n">
         <v>2</v>
       </c>
       <c r="K42" s="11" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="L42" s="10" t="inlineStr">
         <is>
-          <t>T0121</t>
+          <t>T0118</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
         <is>
-          <t>C0045</t>
+          <t>C0043</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>T0077 x T0077</t>
+          <t>T0049 x T0073</t>
         </is>
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Casper</t>
+          <t>Gata</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>14-10-2025</t>
         </is>
       </c>
       <c r="E43" s="11" t="n">
@@ -18262,35 +18496,35 @@
         <v>1</v>
       </c>
       <c r="G43" s="11" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H43" s="11" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J43" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K43" s="11" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="L43" s="10" t="inlineStr">
         <is>
-          <t>T0122</t>
+          <t>T0120</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>C0046</t>
+          <t>C0044</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>T0015 x T0015</t>
+          <t>T0015 x T0067</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
@@ -18300,7 +18534,7 @@
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>16-04-2025</t>
+          <t>03-07-2025</t>
         </is>
       </c>
       <c r="E44" s="11" t="n">
@@ -18310,35 +18544,35 @@
         <v>1</v>
       </c>
       <c r="G44" s="11" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="H44" s="11" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="I44" s="11" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J44" s="11" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K44" s="11" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="L44" s="10" t="inlineStr">
         <is>
-          <t>T0123</t>
+          <t>T0121</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
         <is>
-          <t>C0047</t>
+          <t>C0045</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>T109 x T109</t>
+          <t>T0077 x T0077</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr">
@@ -18348,7 +18582,7 @@
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>12-02-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="E45" s="11" t="n">
@@ -18358,35 +18592,35 @@
         <v>1</v>
       </c>
       <c r="G45" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H45" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I45" s="11" t="n">
         <v>1</v>
       </c>
       <c r="J45" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K45" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L45" s="10" t="inlineStr">
         <is>
-          <t>T0124</t>
+          <t>T0122</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>C0048</t>
+          <t>C0046</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>T0115 x T0115</t>
+          <t>T0015 x T0015</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
@@ -18396,7 +18630,7 @@
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>16-04-2025</t>
         </is>
       </c>
       <c r="E46" s="11" t="n">
@@ -18406,35 +18640,35 @@
         <v>1</v>
       </c>
       <c r="G46" s="11" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="H46" s="11" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="I46" s="11" t="n">
         <v>0</v>
       </c>
       <c r="J46" s="11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K46" s="11" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="L46" s="10" t="inlineStr">
         <is>
-          <t>T0125</t>
+          <t>T0123</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="11" t="inlineStr">
         <is>
-          <t>C0049</t>
+          <t>C0047</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>T0015 x T0114</t>
+          <t>T109 x T109</t>
         </is>
       </c>
       <c r="C47" s="11" t="inlineStr">
@@ -18444,7 +18678,7 @@
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>11-02-2026</t>
+          <t>12-02-2026</t>
         </is>
       </c>
       <c r="E47" s="11" t="n">
@@ -18454,45 +18688,45 @@
         <v>1</v>
       </c>
       <c r="G47" s="11" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="H47" s="11" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="I47" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J47" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K47" s="11" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="L47" s="10" t="inlineStr">
         <is>
-          <t>T0126</t>
+          <t>T0124</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>C0050</t>
+          <t>C0048</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>T0101 x T0101</t>
+          <t>T0115 x T0115</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Gata</t>
+          <t>Casper</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>26-01-2026</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="E48" s="11" t="n">
@@ -18502,35 +18736,35 @@
         <v>1</v>
       </c>
       <c r="G48" s="11" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="H48" s="11" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="I48" s="11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J48" s="11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K48" s="11" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="L48" s="10" t="inlineStr">
         <is>
-          <t>T0127</t>
+          <t>T0125</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
         <is>
-          <t>C0051</t>
+          <t>C0049</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>T0109 x T0115</t>
+          <t>T0015 x T0114</t>
         </is>
       </c>
       <c r="C49" s="11" t="inlineStr">
@@ -18550,10 +18784,10 @@
         <v>1</v>
       </c>
       <c r="G49" s="11" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H49" s="11" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I49" s="11" t="n">
         <v>0</v>
@@ -18562,33 +18796,33 @@
         <v>0</v>
       </c>
       <c r="K49" s="11" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="L49" s="10" t="inlineStr">
         <is>
-          <t>T0131</t>
+          <t>T0126</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>C0052</t>
+          <t>C0050</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>T0082 x T0082</t>
+          <t>T0101 x T0101</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Fli</t>
+          <t>Gata</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>24-11-2025</t>
+          <t>26-01-2026</t>
         </is>
       </c>
       <c r="E50" s="11" t="n">
@@ -18598,45 +18832,45 @@
         <v>1</v>
       </c>
       <c r="G50" s="11" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H50" s="11" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="I50" s="11" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J50" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K50" s="11" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="L50" s="10" t="inlineStr">
         <is>
-          <t>T0133</t>
+          <t>T0127</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
         <is>
-          <t>C0053</t>
+          <t>C0051</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>T0093 x T0101</t>
+          <t>T0109 x T0115</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Gata</t>
+          <t>Casper</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>25-11-2025</t>
+          <t>11-02-2026</t>
         </is>
       </c>
       <c r="E51" s="11" t="n">
@@ -18646,281 +18880,281 @@
         <v>1</v>
       </c>
       <c r="G51" s="11" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H51" s="11" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="J51" s="11" t="n">
         <v>0</v>
       </c>
       <c r="K51" s="11" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="L51" s="10" t="inlineStr">
         <is>
-          <t>T0134</t>
+          <t>T0131</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>C0054</t>
+          <t>C0052</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>T0126 x T0126</t>
+          <t>T0082 x T0082</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Casper</t>
+          <t>Fli</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>29-06-2026</t>
+          <t>24-11-2025</t>
         </is>
       </c>
       <c r="E52" s="11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F52" s="11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G52" s="11" t="n">
-        <v>52</v>
+        <v>11</v>
       </c>
       <c r="H52" s="11" t="n">
-        <v>52</v>
+        <v>11</v>
       </c>
       <c r="I52" s="11" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="J52" s="11" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="K52" s="11" t="n">
-        <v>10.4</v>
+        <v>11</v>
       </c>
       <c r="L52" s="10" t="inlineStr">
         <is>
-          <t>T0135, T0150, T0151, T0156, T0161</t>
+          <t>T0133</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="11" t="inlineStr">
         <is>
-          <t>C0055</t>
+          <t>C0053</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>T0069 x T0069</t>
+          <t>T0093 x T0101</t>
         </is>
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Casper</t>
+          <t>Gata</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>25-11-2025</t>
         </is>
       </c>
       <c r="E53" s="11" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F53" s="11" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G53" s="11" t="n">
-        <v>94</v>
+        <v>14</v>
       </c>
       <c r="H53" s="11" t="n">
-        <v>94</v>
+        <v>14</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="J53" s="11" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K53" s="11" t="n">
-        <v>11.8</v>
+        <v>14</v>
       </c>
       <c r="L53" s="10" t="inlineStr">
         <is>
-          <t>T0136, T0148, T0152, T0154, T0178, T0179, T0180, T0181</t>
+          <t>T0134</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>C0056</t>
+          <t>C0054</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>T0110 x T0110</t>
+          <t>T0126 x T0126</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Gata</t>
+          <t>Casper</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>29-06-2026</t>
         </is>
       </c>
       <c r="E54" s="11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F54" s="11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G54" s="11" t="n">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="H54" s="11" t="n">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="J54" s="11" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="K54" s="11" t="n">
-        <v>15</v>
+        <v>10.4</v>
       </c>
       <c r="L54" s="10" t="inlineStr">
         <is>
-          <t>T0137, T0138</t>
+          <t>T0135, T0150, T0151, T0156, T0161</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
         <is>
-          <t>C0057</t>
-        </is>
-      </c>
-      <c r="B55" s="10" t="inlineStr"/>
+          <t>C0055</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>T0069 x T0069</t>
+        </is>
+      </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Gata</t>
+          <t>Casper</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="E55" s="11" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F55" s="11" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G55" s="11" t="n">
-        <v>15</v>
+        <v>94</v>
       </c>
       <c r="H55" s="11" t="n">
-        <v>15</v>
+        <v>94</v>
       </c>
       <c r="I55" s="11" t="n">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="J55" s="11" t="n">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="K55" s="11" t="n">
-        <v>7.5</v>
+        <v>11.8</v>
       </c>
       <c r="L55" s="10" t="inlineStr">
         <is>
-          <t>T0139, T0140</t>
+          <t>T0136, T0148, T0152, T0154, T0178, T0179, T0180, T0181</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>C0058</t>
+          <t>C0056</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>T0105 x T0056</t>
+          <t>T0110 x T0110</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Fli</t>
+          <t>Gata</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>28-04-2026</t>
+          <t>30-06-2026</t>
         </is>
       </c>
       <c r="E56" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F56" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G56" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="H56" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="I56" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="J56" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="H56" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="I56" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="J56" s="11" t="n">
-        <v>2</v>
-      </c>
       <c r="K56" s="11" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="L56" s="10" t="inlineStr">
         <is>
-          <t>T0141</t>
+          <t>T0137, T0138</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
         <is>
-          <t>C0059</t>
-        </is>
-      </c>
-      <c r="B57" s="10" t="inlineStr">
-        <is>
-          <t>T0123 x T0121</t>
-        </is>
-      </c>
+          <t>C0057</t>
+        </is>
+      </c>
+      <c r="B57" s="10" t="inlineStr"/>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>Casper</t>
+          <t>Gata</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>18-06-2026</t>
+          <t>30-06-2026</t>
         </is>
       </c>
       <c r="E57" s="11" t="n">
@@ -18930,83 +19164,83 @@
         <v>2</v>
       </c>
       <c r="G57" s="11" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="H57" s="11" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="I57" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J57" s="11" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="K57" s="11" t="n">
-        <v>13</v>
+        <v>7.5</v>
       </c>
       <c r="L57" s="10" t="inlineStr">
         <is>
-          <t>T0146, T0147</t>
+          <t>T0139, T0140</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>C0060</t>
+          <t>C0058</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>T0108 x T0108</t>
+          <t>T0105 x T0056</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Casper</t>
+          <t>Fli</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>05-07-2026</t>
+          <t>28-04-2026</t>
         </is>
       </c>
       <c r="E58" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F58" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G58" s="11" t="n">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="H58" s="11" t="n">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="I58" s="11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J58" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K58" s="11" t="n">
-        <v>16.3</v>
+        <v>7</v>
       </c>
       <c r="L58" s="10" t="inlineStr">
         <is>
-          <t>T0149, T0160, T0165</t>
+          <t>T0141</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="11" t="inlineStr">
         <is>
-          <t>C0061</t>
+          <t>C0059</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>T0109 x T0109</t>
+          <t>T0123 x T0121</t>
         </is>
       </c>
       <c r="C59" s="11" t="inlineStr">
@@ -19016,7 +19250,7 @@
       </c>
       <c r="D59" s="11" t="inlineStr">
         <is>
-          <t>14-06-2026</t>
+          <t>18-06-2026</t>
         </is>
       </c>
       <c r="E59" s="11" t="n">
@@ -19026,35 +19260,35 @@
         <v>2</v>
       </c>
       <c r="G59" s="11" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="H59" s="11" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="I59" s="11" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J59" s="11" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="K59" s="11" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="L59" s="10" t="inlineStr">
         <is>
-          <t>T0153, T0163</t>
+          <t>T0146, T0147</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>C0062</t>
+          <t>C0060</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>T0115 x T0115</t>
+          <t>T0108 x T0108</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
@@ -19064,7 +19298,7 @@
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>26-04-2026</t>
+          <t>05-07-2026</t>
         </is>
       </c>
       <c r="E60" s="11" t="n">
@@ -19074,35 +19308,35 @@
         <v>3</v>
       </c>
       <c r="G60" s="11" t="n">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="H60" s="11" t="n">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="I60" s="11" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="J60" s="11" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="K60" s="11" t="n">
-        <v>10</v>
+        <v>16.3</v>
       </c>
       <c r="L60" s="10" t="inlineStr">
         <is>
-          <t>T0157, T0158, T0159</t>
+          <t>T0149, T0160, T0165</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
         <is>
-          <t>C0063</t>
+          <t>C0061</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>T0077 x T0109</t>
+          <t>T0109 x T0109</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
@@ -19116,41 +19350,41 @@
         </is>
       </c>
       <c r="E61" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F61" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G61" s="11" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H61" s="11" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I61" s="11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J61" s="11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K61" s="11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L61" s="10" t="inlineStr">
         <is>
-          <t>T0162</t>
+          <t>T0153, T0163</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>C0064</t>
+          <t>C0062</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>T0122 x T0122</t>
+          <t>T0115 x T0115</t>
         </is>
       </c>
       <c r="C62" s="11" t="inlineStr">
@@ -19160,116 +19394,116 @@
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>15-06-2026</t>
+          <t>26-04-2026</t>
         </is>
       </c>
       <c r="E62" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F62" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G62" s="11" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="H62" s="11" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="I62" s="11" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="J62" s="11" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="K62" s="11" t="n">
         <v>10</v>
       </c>
       <c r="L62" s="10" t="inlineStr">
         <is>
-          <t>T0164</t>
+          <t>T0157, T0158, T0159</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="inlineStr">
         <is>
-          <t>C0065</t>
+          <t>C0063</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>T0081 x T0081</t>
+          <t>T0077 x T0109</t>
         </is>
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>AB</t>
+          <t>Casper</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr">
         <is>
-          <t>12-05-2026</t>
+          <t>14-06-2026</t>
         </is>
       </c>
       <c r="E63" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F63" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G63" s="11" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="H63" s="11" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="I63" s="11" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="J63" s="11" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K63" s="11" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="L63" s="10" t="inlineStr">
         <is>
-          <t>T0166, T0167</t>
+          <t>T0162</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>C0067</t>
+          <t>C0064</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>T0098 x T0133</t>
+          <t>T0122 x T0122</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Fli</t>
+          <t>Casper</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>17-08-2026</t>
+          <t>15-06-2026</t>
         </is>
       </c>
       <c r="E64" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F64" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G64" s="11" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="H64" s="11" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="I64" s="11" t="n">
         <v>0</v>
@@ -19278,71 +19512,71 @@
         <v>0</v>
       </c>
       <c r="K64" s="11" t="n">
-        <v>27.5</v>
+        <v>10</v>
       </c>
       <c r="L64" s="10" t="inlineStr">
         <is>
-          <t>T0171, T0172</t>
+          <t>T0164</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
         <is>
-          <t>C0068</t>
+          <t>C0065</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>T0119 x T0119</t>
+          <t>T0081 x T0081</t>
         </is>
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Fli</t>
+          <t>AB</t>
         </is>
       </c>
       <c r="D65" s="11" t="inlineStr">
         <is>
-          <t>16-08-2026</t>
+          <t>12-05-2026</t>
         </is>
       </c>
       <c r="E65" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F65" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G65" s="11" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="H65" s="11" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="I65" s="11" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="J65" s="11" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K65" s="11" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="L65" s="10" t="inlineStr">
         <is>
-          <t>T0173</t>
+          <t>T0166, T0167</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>C0069</t>
+          <t>C0067</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>T0133 x T0133</t>
+          <t>T0098 x T0133</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr">
@@ -19356,16 +19590,16 @@
         </is>
       </c>
       <c r="E66" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F66" s="11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G66" s="11" t="n">
-        <v>9</v>
+        <v>55</v>
       </c>
       <c r="H66" s="11" t="n">
-        <v>9</v>
+        <v>55</v>
       </c>
       <c r="I66" s="11" t="n">
         <v>0</v>
@@ -19374,23 +19608,23 @@
         <v>0</v>
       </c>
       <c r="K66" s="11" t="n">
-        <v>9</v>
+        <v>27.5</v>
       </c>
       <c r="L66" s="10" t="inlineStr">
         <is>
-          <t>T0174</t>
+          <t>T0171, T0172</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="11" t="inlineStr">
         <is>
-          <t>C0070</t>
+          <t>C0068</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>T0132 x T0132</t>
+          <t>T0119 x T0119</t>
         </is>
       </c>
       <c r="C67" s="11" t="inlineStr">
@@ -19404,41 +19638,41 @@
         </is>
       </c>
       <c r="E67" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F67" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G67" s="11" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="H67" s="11" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="I67" s="11" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J67" s="11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K67" s="11" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="L67" s="10" t="inlineStr">
         <is>
-          <t>T0175, T0176</t>
+          <t>T0173</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>C0071</t>
+          <t>C0069</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>T0082 x T0082</t>
+          <t>T0133 x T0133</t>
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr">
@@ -19448,7 +19682,7 @@
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>07-04-2026</t>
+          <t>17-08-2026</t>
         </is>
       </c>
       <c r="E68" s="11" t="n">
@@ -19458,21 +19692,117 @@
         <v>1</v>
       </c>
       <c r="G68" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="H68" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="I68" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="L68" s="10" t="inlineStr">
+        <is>
+          <t>T0174</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>C0070</t>
+        </is>
+      </c>
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t>T0132 x T0132</t>
+        </is>
+      </c>
+      <c r="C69" s="11" t="inlineStr">
+        <is>
+          <t>Fli</t>
+        </is>
+      </c>
+      <c r="D69" s="11" t="inlineStr">
+        <is>
+          <t>16-08-2026</t>
+        </is>
+      </c>
+      <c r="E69" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F69" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G69" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="H69" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="I69" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="J69" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="K69" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="H68" s="11" t="n">
+      <c r="L69" s="10" t="inlineStr">
+        <is>
+          <t>T0175, T0176</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>C0071</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="inlineStr">
+        <is>
+          <t>T0082 x T0082</t>
+        </is>
+      </c>
+      <c r="C70" s="11" t="inlineStr">
+        <is>
+          <t>Fli</t>
+        </is>
+      </c>
+      <c r="D70" s="11" t="inlineStr">
+        <is>
+          <t>07-04-2026</t>
+        </is>
+      </c>
+      <c r="E70" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="I68" s="11" t="n">
+      <c r="H70" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="I70" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="J68" s="11" t="n">
+      <c r="J70" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="K68" s="11" t="n">
+      <c r="K70" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="L68" s="10" t="inlineStr">
+      <c r="L70" s="10" t="inlineStr">
         <is>
           <t>T0177</t>
         </is>
@@ -19489,7 +19819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:J124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -24950,6 +25280,124 @@
       <c r="J121" s="17" t="inlineStr">
         <is>
           <t>Consider consolidating or moving to 1.8L tank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="11" t="inlineStr"/>
+      <c r="B122" s="11" t="inlineStr">
+        <is>
+          <t>Adult/Active</t>
+        </is>
+      </c>
+      <c r="C122" s="10" t="inlineStr"/>
+      <c r="D122" s="11" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E122" s="11" t="inlineStr"/>
+      <c r="F122" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G122" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I122" s="11" t="inlineStr">
+        <is>
+          <t>Empty / Unknown</t>
+        </is>
+      </c>
+      <c r="J122" s="10" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="11" t="inlineStr">
+        <is>
+          <t>10-08-26</t>
+        </is>
+      </c>
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>Adult/Active</t>
+        </is>
+      </c>
+      <c r="C123" s="10" t="inlineStr"/>
+      <c r="D123" s="11" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E123" s="11" t="inlineStr">
+        <is>
+          <t>Wt (AB)</t>
+        </is>
+      </c>
+      <c r="F123" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G123" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="H123" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I123" s="11" t="inlineStr">
+        <is>
+          <t>Empty / Unknown</t>
+        </is>
+      </c>
+      <c r="J123" s="10" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="11" t="inlineStr">
+        <is>
+          <t>10-08-26</t>
+        </is>
+      </c>
+      <c r="B124" s="11" t="inlineStr">
+        <is>
+          <t>Adult/Active</t>
+        </is>
+      </c>
+      <c r="C124" s="10" t="inlineStr"/>
+      <c r="D124" s="11" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E124" s="11" t="inlineStr">
+        <is>
+          <t>Wt (AB)</t>
+        </is>
+      </c>
+      <c r="F124" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G124" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="H124" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I124" s="11" t="inlineStr">
+        <is>
+          <t>Empty / Unknown</t>
+        </is>
+      </c>
+      <c r="J124" s="10" t="inlineStr">
+        <is>
+          <t>Compliant</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix inventory table schema, tank count (183 tanks), restore FileMaker columns & remove non-functional web ingestion
</commit_message>
<xml_diff>
--- a/FishNET_Colony_Analytics_Report.xlsx
+++ b/FishNET_Colony_Analytics_Report.xlsx
@@ -569,14 +569,14 @@
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Total Recorded Tanks
-182</t>
+183</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Active Holding Tanks
-182</t>
+183</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C13" s="10" t="n">
         <v>0</v>
@@ -1310,7 +1310,7 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>0</v>
@@ -1357,7 +1357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M186"/>
+  <dimension ref="A1:M187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8919,6 +8919,47 @@
         </is>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" s="13" t="inlineStr">
+        <is>
+          <t>T0184</t>
+        </is>
+      </c>
+      <c r="B187" s="13" t="inlineStr">
+        <is>
+          <t>Adult/Active</t>
+        </is>
+      </c>
+      <c r="C187" s="12" t="inlineStr"/>
+      <c r="D187" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E187" s="13" t="inlineStr"/>
+      <c r="F187" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G187" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H187" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I187" s="13" t="inlineStr"/>
+      <c r="J187" s="13" t="inlineStr"/>
+      <c r="K187" s="13" t="n"/>
+      <c r="L187" s="13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="M187" s="12" t="inlineStr">
+        <is>
+          <t>Inactive or No turnover date set.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8930,7 +8971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K186"/>
+  <dimension ref="A1:K187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -14295,6 +14336,35 @@
       </c>
       <c r="J186" s="12" t="inlineStr"/>
       <c r="K186" s="12" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="13" t="inlineStr">
+        <is>
+          <t>T0184</t>
+        </is>
+      </c>
+      <c r="B187" s="13" t="inlineStr"/>
+      <c r="C187" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D187" s="13" t="inlineStr">
+        <is>
+          <t>F0 / Founder</t>
+        </is>
+      </c>
+      <c r="E187" s="13" t="inlineStr"/>
+      <c r="F187" s="13" t="inlineStr"/>
+      <c r="G187" s="13" t="inlineStr"/>
+      <c r="H187" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I187" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J187" s="12" t="inlineStr"/>
+      <c r="K187" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14412,7 +14482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J186"/>
+  <dimension ref="A1:J187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -21405,6 +21475,44 @@
         </is>
       </c>
       <c r="J186" s="12" t="inlineStr">
+        <is>
+          <t>Compliant</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="13" t="inlineStr">
+        <is>
+          <t>T0184</t>
+        </is>
+      </c>
+      <c r="B187" s="13" t="inlineStr">
+        <is>
+          <t>Adult/Active</t>
+        </is>
+      </c>
+      <c r="C187" s="12" t="inlineStr"/>
+      <c r="D187" s="13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E187" s="13" t="inlineStr"/>
+      <c r="F187" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G187" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H187" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I187" s="13" t="inlineStr">
+        <is>
+          <t>Empty / Unknown</t>
+        </is>
+      </c>
+      <c r="J187" s="12" t="inlineStr">
         <is>
           <t>Compliant</t>
         </is>

</xml_diff>

<commit_message>
Update facility standards: 18-month turnover policy (540 days) and optimal 5.0 fish/L stocking density
</commit_message>
<xml_diff>
--- a/FishNET_Colony_Analytics_Report.xlsx
+++ b/FishNET_Colony_Analytics_Report.xlsx
@@ -16500,8 +16500,8 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="43" customWidth="1" min="9" max="9"/>
-    <col width="49" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="54" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16514,7 +16514,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Active tanks density evaluation (Target: 2.0 - 6.0 fish/L. Welfare threshold: &lt; 8.0 fish/L).</t>
+          <t>Active tanks density evaluation (Target: 1.0 - 5.0 fish/L. Welfare threshold: &lt;= 7.0 fish/L).</t>
         </is>
       </c>
     </row>
@@ -16572,94 +16572,94 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>T0171</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>Adult/Active</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Adult/Active</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>Fli T133 x Fli T98 (1)</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Fli</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>3.8L</t>
         </is>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="13" t="n">
         <v>3.8</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G5" s="13" t="n">
         <v>28</v>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="H5" s="13" t="n">
         <v>7.37</v>
       </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>Moderate / Acceptable (6.1 - 8.0 fish/L)</t>
-        </is>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
-        <is>
-          <t>Compliant</t>
+      <c r="I5" s="13" t="inlineStr">
+        <is>
+          <t>OVERSTOCKED (&gt;7.0 fish/L - Welfare Alert)</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Split tank immediately into secondary holding tank.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>T0172</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Adult/Active</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Adult/Active</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>Fli T133 x Fli T98 (2)</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Fli</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>3.8L</t>
         </is>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="13" t="n">
         <v>3.8</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="G6" s="13" t="n">
         <v>27</v>
       </c>
-      <c r="H6" s="11" t="n">
+      <c r="H6" s="13" t="n">
         <v>7.11</v>
       </c>
-      <c r="I6" s="11" t="inlineStr">
-        <is>
-          <t>Moderate / Acceptable (6.1 - 8.0 fish/L)</t>
-        </is>
-      </c>
-      <c r="J6" s="10" t="inlineStr">
-        <is>
-          <t>Compliant</t>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>OVERSTOCKED (&gt;7.0 fish/L - Welfare Alert)</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Split tank immediately into secondary holding tank.</t>
         </is>
       </c>
     </row>
@@ -16700,7 +16700,7 @@
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>Moderate / Acceptable (6.1 - 8.0 fish/L)</t>
+          <t>Moderate (5.1 - 7.0 fish/L)</t>
         </is>
       </c>
       <c r="J7" s="10" t="inlineStr">
@@ -16746,7 +16746,7 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Moderate / Acceptable (6.1 - 8.0 fish/L)</t>
+          <t>Moderate (5.1 - 7.0 fish/L)</t>
         </is>
       </c>
       <c r="J8" s="10" t="inlineStr">
@@ -16792,7 +16792,7 @@
       </c>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Moderate (5.1 - 7.0 fish/L)</t>
         </is>
       </c>
       <c r="J9" s="10" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Moderate (5.1 - 7.0 fish/L)</t>
         </is>
       </c>
       <c r="J10" s="10" t="inlineStr">
@@ -16884,7 +16884,7 @@
       </c>
       <c r="I11" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Moderate (5.1 - 7.0 fish/L)</t>
         </is>
       </c>
       <c r="J11" s="10" t="inlineStr">
@@ -16930,7 +16930,7 @@
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Moderate (5.1 - 7.0 fish/L)</t>
         </is>
       </c>
       <c r="J12" s="10" t="inlineStr">
@@ -16976,7 +16976,7 @@
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Moderate (5.1 - 7.0 fish/L)</t>
         </is>
       </c>
       <c r="J13" s="10" t="inlineStr">
@@ -17022,7 +17022,7 @@
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Moderate (5.1 - 7.0 fish/L)</t>
         </is>
       </c>
       <c r="J14" s="10" t="inlineStr">
@@ -17068,7 +17068,7 @@
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J15" s="10" t="inlineStr">
@@ -17114,7 +17114,7 @@
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J16" s="10" t="inlineStr">
@@ -17160,7 +17160,7 @@
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J17" s="10" t="inlineStr">
@@ -17206,7 +17206,7 @@
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J18" s="10" t="inlineStr">
@@ -17252,7 +17252,7 @@
       </c>
       <c r="I19" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J19" s="10" t="inlineStr">
@@ -17298,7 +17298,7 @@
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J20" s="10" t="inlineStr">
@@ -17344,7 +17344,7 @@
       </c>
       <c r="I21" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J21" s="10" t="inlineStr">
@@ -17390,7 +17390,7 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J22" s="10" t="inlineStr">
@@ -17436,7 +17436,7 @@
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J23" s="10" t="inlineStr">
@@ -17482,7 +17482,7 @@
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J24" s="10" t="inlineStr">
@@ -17528,7 +17528,7 @@
       </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J25" s="10" t="inlineStr">
@@ -17574,7 +17574,7 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J26" s="10" t="inlineStr">
@@ -17620,7 +17620,7 @@
       </c>
       <c r="I27" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J27" s="10" t="inlineStr">
@@ -17666,7 +17666,7 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J28" s="10" t="inlineStr">
@@ -17712,7 +17712,7 @@
       </c>
       <c r="I29" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J29" s="10" t="inlineStr">
@@ -17758,7 +17758,7 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J30" s="10" t="inlineStr">
@@ -17804,7 +17804,7 @@
       </c>
       <c r="I31" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J31" s="10" t="inlineStr">
@@ -17850,7 +17850,7 @@
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J32" s="10" t="inlineStr">
@@ -17896,7 +17896,7 @@
       </c>
       <c r="I33" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J33" s="10" t="inlineStr">
@@ -17942,7 +17942,7 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J34" s="10" t="inlineStr">
@@ -17988,7 +17988,7 @@
       </c>
       <c r="I35" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J35" s="10" t="inlineStr">
@@ -18034,7 +18034,7 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J36" s="10" t="inlineStr">
@@ -18080,7 +18080,7 @@
       </c>
       <c r="I37" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J37" s="10" t="inlineStr">
@@ -18126,7 +18126,7 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J38" s="10" t="inlineStr">
@@ -18172,7 +18172,7 @@
       </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J39" s="10" t="inlineStr">
@@ -18218,7 +18218,7 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J40" s="10" t="inlineStr">
@@ -18264,7 +18264,7 @@
       </c>
       <c r="I41" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J41" s="10" t="inlineStr">
@@ -18310,7 +18310,7 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J42" s="10" t="inlineStr">
@@ -18356,7 +18356,7 @@
       </c>
       <c r="I43" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J43" s="10" t="inlineStr">
@@ -18402,7 +18402,7 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J44" s="10" t="inlineStr">
@@ -18448,7 +18448,7 @@
       </c>
       <c r="I45" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J45" s="10" t="inlineStr">
@@ -18494,7 +18494,7 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J46" s="10" t="inlineStr">
@@ -18540,7 +18540,7 @@
       </c>
       <c r="I47" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J47" s="10" t="inlineStr">
@@ -18586,7 +18586,7 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J48" s="10" t="inlineStr">
@@ -18632,7 +18632,7 @@
       </c>
       <c r="I49" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J49" s="10" t="inlineStr">
@@ -18678,7 +18678,7 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J50" s="10" t="inlineStr">
@@ -18724,7 +18724,7 @@
       </c>
       <c r="I51" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J51" s="10" t="inlineStr">
@@ -18770,7 +18770,7 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J52" s="10" t="inlineStr">
@@ -18816,7 +18816,7 @@
       </c>
       <c r="I53" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J53" s="10" t="inlineStr">
@@ -18862,7 +18862,7 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J54" s="10" t="inlineStr">
@@ -18908,7 +18908,7 @@
       </c>
       <c r="I55" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J55" s="10" t="inlineStr">
@@ -18954,7 +18954,7 @@
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J56" s="10" t="inlineStr">
@@ -19000,7 +19000,7 @@
       </c>
       <c r="I57" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J57" s="10" t="inlineStr">
@@ -19046,7 +19046,7 @@
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J58" s="10" t="inlineStr">
@@ -19092,7 +19092,7 @@
       </c>
       <c r="I59" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J59" s="10" t="inlineStr">
@@ -19138,7 +19138,7 @@
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J60" s="10" t="inlineStr">
@@ -19184,7 +19184,7 @@
       </c>
       <c r="I61" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J61" s="10" t="inlineStr">
@@ -19230,7 +19230,7 @@
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J62" s="10" t="inlineStr">
@@ -19276,7 +19276,7 @@
       </c>
       <c r="I63" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J63" s="10" t="inlineStr">
@@ -19322,7 +19322,7 @@
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J64" s="10" t="inlineStr">
@@ -19368,7 +19368,7 @@
       </c>
       <c r="I65" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J65" s="10" t="inlineStr">
@@ -19414,7 +19414,7 @@
       </c>
       <c r="I66" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J66" s="10" t="inlineStr">
@@ -19460,7 +19460,7 @@
       </c>
       <c r="I67" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J67" s="10" t="inlineStr">
@@ -19506,7 +19506,7 @@
       </c>
       <c r="I68" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J68" s="10" t="inlineStr">
@@ -19552,7 +19552,7 @@
       </c>
       <c r="I69" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J69" s="10" t="inlineStr">
@@ -19598,7 +19598,7 @@
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J70" s="10" t="inlineStr">
@@ -19644,7 +19644,7 @@
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J71" s="10" t="inlineStr">
@@ -19690,7 +19690,7 @@
       </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J72" s="10" t="inlineStr">
@@ -19736,7 +19736,7 @@
       </c>
       <c r="I73" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J73" s="10" t="inlineStr">
@@ -19782,7 +19782,7 @@
       </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J74" s="10" t="inlineStr">
@@ -19828,7 +19828,7 @@
       </c>
       <c r="I75" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J75" s="10" t="inlineStr">
@@ -19874,7 +19874,7 @@
       </c>
       <c r="I76" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J76" s="10" t="inlineStr">
@@ -19920,7 +19920,7 @@
       </c>
       <c r="I77" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J77" s="10" t="inlineStr">
@@ -19966,7 +19966,7 @@
       </c>
       <c r="I78" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J78" s="10" t="inlineStr">
@@ -20012,7 +20012,7 @@
       </c>
       <c r="I79" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J79" s="10" t="inlineStr">
@@ -20058,7 +20058,7 @@
       </c>
       <c r="I80" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J80" s="10" t="inlineStr">
@@ -20104,7 +20104,7 @@
       </c>
       <c r="I81" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J81" s="10" t="inlineStr">
@@ -20150,7 +20150,7 @@
       </c>
       <c r="I82" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J82" s="10" t="inlineStr">
@@ -20196,7 +20196,7 @@
       </c>
       <c r="I83" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J83" s="10" t="inlineStr">
@@ -20242,7 +20242,7 @@
       </c>
       <c r="I84" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J84" s="10" t="inlineStr">
@@ -20288,7 +20288,7 @@
       </c>
       <c r="I85" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J85" s="10" t="inlineStr">
@@ -20334,7 +20334,7 @@
       </c>
       <c r="I86" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J86" s="10" t="inlineStr">
@@ -20380,7 +20380,7 @@
       </c>
       <c r="I87" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J87" s="10" t="inlineStr">
@@ -20426,7 +20426,7 @@
       </c>
       <c r="I88" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J88" s="10" t="inlineStr">
@@ -20472,7 +20472,7 @@
       </c>
       <c r="I89" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J89" s="10" t="inlineStr">
@@ -20518,7 +20518,7 @@
       </c>
       <c r="I90" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J90" s="10" t="inlineStr">
@@ -20564,7 +20564,7 @@
       </c>
       <c r="I91" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J91" s="10" t="inlineStr">
@@ -20610,7 +20610,7 @@
       </c>
       <c r="I92" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J92" s="10" t="inlineStr">
@@ -20656,7 +20656,7 @@
       </c>
       <c r="I93" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J93" s="10" t="inlineStr">
@@ -20702,7 +20702,7 @@
       </c>
       <c r="I94" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J94" s="10" t="inlineStr">
@@ -20748,7 +20748,7 @@
       </c>
       <c r="I95" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J95" s="10" t="inlineStr">
@@ -20794,7 +20794,7 @@
       </c>
       <c r="I96" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J96" s="10" t="inlineStr">
@@ -20840,7 +20840,7 @@
       </c>
       <c r="I97" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J97" s="10" t="inlineStr">
@@ -20886,7 +20886,7 @@
       </c>
       <c r="I98" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J98" s="10" t="inlineStr">
@@ -20932,7 +20932,7 @@
       </c>
       <c r="I99" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J99" s="10" t="inlineStr">
@@ -20978,7 +20978,7 @@
       </c>
       <c r="I100" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J100" s="10" t="inlineStr">
@@ -21024,7 +21024,7 @@
       </c>
       <c r="I101" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J101" s="10" t="inlineStr">
@@ -21070,7 +21070,7 @@
       </c>
       <c r="I102" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J102" s="10" t="inlineStr">
@@ -21116,7 +21116,7 @@
       </c>
       <c r="I103" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J103" s="10" t="inlineStr">
@@ -21162,7 +21162,7 @@
       </c>
       <c r="I104" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J104" s="10" t="inlineStr">
@@ -21208,7 +21208,7 @@
       </c>
       <c r="I105" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J105" s="10" t="inlineStr">
@@ -21254,7 +21254,7 @@
       </c>
       <c r="I106" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J106" s="10" t="inlineStr">
@@ -21300,7 +21300,7 @@
       </c>
       <c r="I107" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J107" s="10" t="inlineStr">
@@ -21346,7 +21346,7 @@
       </c>
       <c r="I108" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J108" s="10" t="inlineStr">
@@ -21392,7 +21392,7 @@
       </c>
       <c r="I109" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J109" s="10" t="inlineStr">
@@ -21438,7 +21438,7 @@
       </c>
       <c r="I110" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J110" s="10" t="inlineStr">
@@ -21484,7 +21484,7 @@
       </c>
       <c r="I111" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J111" s="10" t="inlineStr">
@@ -21530,7 +21530,7 @@
       </c>
       <c r="I112" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J112" s="10" t="inlineStr">
@@ -21576,7 +21576,7 @@
       </c>
       <c r="I113" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J113" s="10" t="inlineStr">
@@ -21622,7 +21622,7 @@
       </c>
       <c r="I114" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J114" s="10" t="inlineStr">
@@ -21668,7 +21668,7 @@
       </c>
       <c r="I115" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J115" s="10" t="inlineStr">
@@ -21714,7 +21714,7 @@
       </c>
       <c r="I116" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J116" s="10" t="inlineStr">
@@ -21760,7 +21760,7 @@
       </c>
       <c r="I117" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J117" s="10" t="inlineStr">
@@ -21806,7 +21806,7 @@
       </c>
       <c r="I118" s="11" t="inlineStr">
         <is>
-          <t>Optimal (1.0 - 6.0 fish/L)</t>
+          <t>Optimal (1.0 - 5.0 fish/L)</t>
         </is>
       </c>
       <c r="J118" s="10" t="inlineStr">
@@ -22102,7 +22102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -22124,7 +22124,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Active Actionable Alerts: 76</t>
+          <t>Total Active Actionable Alerts: 78</t>
         </is>
       </c>
     </row>
@@ -24975,6 +24975,80 @@
       <c r="G80" s="10" t="inlineStr">
         <is>
           <t>Identify compatible female tank for future crosses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>ALT-077</t>
+        </is>
+      </c>
+      <c r="B81" s="14" t="inlineStr">
+        <is>
+          <t>T0171</t>
+        </is>
+      </c>
+      <c r="C81" s="14" t="inlineStr">
+        <is>
+          <t>Fli</t>
+        </is>
+      </c>
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>Animal Welfare (Density)</t>
+        </is>
+      </c>
+      <c r="E81" s="14" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F81" s="15" t="inlineStr">
+        <is>
+          <t>High stocking density: 7.37 fish/L in a 3.8L tank (28 fish).</t>
+        </is>
+      </c>
+      <c r="G81" s="15" t="inlineStr">
+        <is>
+          <t>Split stock into two tanks to maintain 4-6 fish/L welfare guidelines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>ALT-078</t>
+        </is>
+      </c>
+      <c r="B82" s="14" t="inlineStr">
+        <is>
+          <t>T0172</t>
+        </is>
+      </c>
+      <c r="C82" s="14" t="inlineStr">
+        <is>
+          <t>Fli</t>
+        </is>
+      </c>
+      <c r="D82" s="15" t="inlineStr">
+        <is>
+          <t>Animal Welfare (Density)</t>
+        </is>
+      </c>
+      <c r="E82" s="14" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F82" s="15" t="inlineStr">
+        <is>
+          <t>High stocking density: 7.11 fish/L in a 3.8L tank (27 fish).</t>
+        </is>
+      </c>
+      <c r="G82" s="15" t="inlineStr">
+        <is>
+          <t>Split stock into two tanks to maintain 4-6 fish/L welfare guidelines.</t>
         </is>
       </c>
     </row>

</xml_diff>